<commit_message>
chore: sync user words into Excel and vocab-data
</commit_message>
<xml_diff>
--- a/docs/interview-vocab.xlsx
+++ b/docs/interview-vocab.xlsx
@@ -59306,7 +59306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59520,89 +59520,89 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>社区·JavaScript常用单词</t>
+          <t>社区·深度学习 · AI / 其他</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>debounce</t>
+          <t>checkpoint</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>防抖函数</t>
+          <t>某一时刻保存的模型权重。</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>迪邦斯</t>
+          <t>切克点特</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>/dibauns/</t>
+          <t>/ˈtʃekpɔɪnt/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>/dibauns/</t>
+          <t>/ˈtʃekpɔɪnt/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>AI / 其他</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>了解</t>
+          <t>常问</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Debounce / Throttle</t>
+          <t>save / resume</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>防抖函数。</t>
+          <t>按验证集最优存盘，方便回滚和续训。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>社区投稿</t>
+          <t>社区·JavaScript常用单词</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>delete</t>
+          <t>debounce</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>delete：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>防抖函数</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>德-诶-勒-诶-特-诶</t>
+          <t>迪邦斯</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>/dɪˈliːt/</t>
+          <t>/dibauns/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>delete</t>
+          <t>/dibauns/</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>通用</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -59612,44 +59612,44 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Debounce / Throttle</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>一句话：delete：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>防抖函数。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>社区·未分类</t>
+          <t>社区投稿</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>example</t>
+          <t>delete</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>平行或非常相似的案例，特别是作为先例或模型时。</t>
+          <t>delete：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>伊-格-兹-阿-姆-普-勒</t>
+          <t>德-诶-勒-诶-特-诶</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>/ɪɡˈzɑːmpl̩/</t>
+          <t>/dɪˈliːt/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>/ɪɡˈzɑːmpl̩/</t>
+          <t>delete</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -59669,39 +59669,39 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>平行或非常相似的案例，特别是作为先例或模型时。</t>
+          <t>一句话：delete：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>社区投稿</t>
+          <t>社区·未分类</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>for</t>
+          <t>example</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>for：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>平行或非常相似的案例，特别是作为先例或模型时。</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>弗-尔</t>
+          <t>伊-格-兹-阿-姆-普-勒</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>英 /fɔː(r); fə(r)/  美 /fɔːr; fər/</t>
+          <t>/ɪɡˈzɑːmpl̩/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>for</t>
+          <t>/ɪɡˈzɑːmpl̩/</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -59721,7 +59721,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>一句话：for：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>平行或非常相似的案例，特别是作为先例或模型时。</t>
         </is>
       </c>
     </row>
@@ -59733,23 +59733,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>idemmode</t>
+          <t>for</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>idemmode：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>for：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>伊-德-诶-姆-姆-德-诶</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>弗-尔</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>英 /fɔː(r); fə(r)/  美 /fɔːr; fər/</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>idemmode</t>
+          <t>for</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -59769,39 +59773,35 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>一句话：idemmode：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>一句话：for：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>社区·未分类</t>
+          <t>社区投稿</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>idepment</t>
+          <t>idemmode</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>idepment：面试中需能解释其含义，并结合项目说明使用场景。</t>
+          <t>idemmode：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>伊-德-伊-普-门特</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>/ɪdepmənt/</t>
-        </is>
-      </c>
+          <t>伊-德-诶-姆-姆-德-诶</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>/ɪdepmənt/</t>
+          <t>idemmode</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -59821,39 +59821,39 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>能说明 idepment 的含义，并举例它在项目中的用法。</t>
+          <t>一句话：idemmode：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>社区投稿</t>
+          <t>社区·未分类</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IS</t>
+          <t>idepment</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>IS：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>idepment：面试中需能解释其含义，并结合项目说明使用场景。</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>伊-斯</t>
+          <t>伊-德-伊-普-门特</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>/ɪz/</t>
+          <t>/ɪdepmənt/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>IS</t>
+          <t>/ɪdepmənt/</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -59873,7 +59873,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>一句话：IS：技术面试常见术语，建议结合项目场景理解。</t>
+          <t>能说明 idepment 的含义，并举例它在项目中的用法。</t>
         </is>
       </c>
     </row>
@@ -59885,27 +59885,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pink</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>常见的小鱼， Phoxinus phoxinus。</t>
+          <t>IS：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>普-伊-恩-克</t>
+          <t>伊-斯</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/pɪŋk/</t>
+          <t>/ɪz/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>pink</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -59925,109 +59925,161 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>一句话：常见的小鱼， Phoxinus phoxinus。</t>
+          <t>一句话：IS：技术面试常见术语，建议结合项目场景理解。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>社区·基础 · AI</t>
+          <t>社区投稿</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>prompt</t>
+          <t>pink</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>提示词，引导模型输出</t>
+          <t>常见的小鱼， Phoxinus phoxinus。</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>普-罗姆普特</t>
+          <t>普-伊-恩-克</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/prɒmpt/</t>
+          <t>/pɪŋk/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>/prɒmpt/</t>
+          <t>pink</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>必问</t>
+          <t>了解</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>System / Few-shot</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>引导模型输出的指令和上下文。</t>
+          <t>一句话：常见的小鱼， Phoxinus phoxinus。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>社区·基础 · AI</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>prompt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>提示词，引导模型输出</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>普-罗姆普特</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>/prɒmpt/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>/prɒmpt/</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>必问</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>System / Few-shot</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>引导模型输出的指令和上下文。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>社区·未分类</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Reconciliation</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Reconciliation：面试中需能解释其含义，并结合项目说明使用场景。</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>尔-诶-克-奥-恩-克-伊-勒-伊-阿-什-呃-恩</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>/rekɒnkɪlɪæʃən/</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>/rekɒnkɪlɪæʃən/</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>通用</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>了解</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>能说明 Reconciliation 的含义，并举例它在项目中的用法。</t>
         </is>

</xml_diff>